<commit_message>
Add air foil bearing, rotor structure, cooling passage categories to patent template
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kf9BGN4Y1VnhTqa88N2gbo
</commit_message>
<xml_diff>
--- a/특허_주간정리_양식.xlsx
+++ b/특허_주간정리_양식.xlsx
@@ -147,7 +147,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">베어링 </t>
+          <t xml:space="preserve">에어포일 베어링 </t>
         </r>
         <r>
           <rPr>
@@ -156,6 +156,166 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">/ </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">기타 베어링</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">자기</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">·</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">볼 등</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">) / </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">회전체 구조</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">로터</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">·</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">축</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">·</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">임펠러 체결</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">·</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">로터다이내믹스</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">) / </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">모터 </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">/ </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="WenQuanYi Zen Hei"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">냉각유로</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">(</t>
         </r>
         <r>
           <rPr>
@@ -179,7 +339,7 @@
             <rFont val="WenQuanYi Zen Hei"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">로터 </t>
+          <t xml:space="preserve">베어링 냉각 유로</t>
         </r>
         <r>
           <rPr>
@@ -187,23 +347,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">/ </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="WenQuanYi Zen Hei"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">냉각 </t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">/ </t>
+          <t xml:space="preserve">) / </t>
         </r>
         <r>
           <rPr>
@@ -328,7 +472,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="80">
   <si>
     <r>
       <rPr>
@@ -447,7 +591,19 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">베어링</t>
+    <t xml:space="preserve">에어포일 베어링</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기타 베어링</t>
+  </si>
+  <si>
+    <t xml:space="preserve">회전체 구조</t>
+  </si>
+  <si>
+    <t xml:space="preserve">모터</t>
+  </si>
+  <si>
+    <t xml:space="preserve">냉각유로</t>
   </si>
   <si>
     <r>
@@ -458,7 +614,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">모터</t>
+      <t xml:space="preserve">제어</t>
     </r>
     <r>
       <rPr>
@@ -479,11 +635,17 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">로터</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">냉각</t>
+      <t xml:space="preserve">서지</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">시스템</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기타</t>
+  </si>
+  <si>
+    <t xml:space="preserve">합계</t>
   </si>
   <si>
     <r>
@@ -494,7 +656,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">제어</t>
+      <t xml:space="preserve">중요도 </t>
     </r>
     <r>
       <rPr>
@@ -505,7 +667,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">·</t>
+      <t xml:space="preserve">'</t>
     </r>
     <r>
       <rPr>
@@ -515,150 +677,159 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">서지</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">시스템</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기타</t>
-  </si>
-  <si>
-    <t xml:space="preserve">합계</t>
-  </si>
-  <si>
+      <t xml:space="preserve">상</t>
+    </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">중요도 </t>
-    </r>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">LG</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">전자</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">댄포스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">코플랜드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">덴소</t>
+  </si>
+  <si>
+    <t xml:space="preserve">다이킨</t>
+  </si>
+  <si>
+    <t xml:space="preserve">티앤이코리아</t>
+  </si>
+  <si>
+    <t xml:space="preserve">터보맥스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보고일</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">출원인</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">상</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">LG</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">전자</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">댄포스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">코플랜드</t>
-  </si>
-  <si>
-    <t xml:space="preserve">덴소</t>
-  </si>
-  <si>
-    <t xml:space="preserve">다이킨</t>
-  </si>
-  <si>
-    <t xml:space="preserve">티앤이코리아</t>
-  </si>
-  <si>
-    <t xml:space="preserve">터보맥스</t>
-  </si>
-  <si>
-    <t xml:space="preserve">보고일</t>
-  </si>
-  <si>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원문</t>
+    </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">출원인</t>
-    </r>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">국가</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공개</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">원문</t>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
     </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">국가</t>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">등록번호</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">구분</t>
+  </si>
+  <si>
+    <t xml:space="preserve">제목</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공개일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">출원일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">설계 분야</t>
+  </si>
+  <si>
+    <t xml:space="preserve">용도</t>
   </si>
   <si>
     <r>
@@ -669,7 +840,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">공개</t>
+      <t xml:space="preserve">핵심 내용</t>
     </r>
     <r>
       <rPr>
@@ -680,7 +851,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">/</t>
+      <t xml:space="preserve">(</t>
     </r>
     <r>
       <rPr>
@@ -690,64 +861,13 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">등록번호</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">구분</t>
-  </si>
-  <si>
-    <t xml:space="preserve">제목</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공개일</t>
-  </si>
-  <si>
-    <t xml:space="preserve">출원일</t>
-  </si>
-  <si>
-    <t xml:space="preserve">설계 분야</t>
-  </si>
-  <si>
-    <t xml:space="preserve">용도</t>
-  </si>
-  <si>
+      <t xml:space="preserve">설계 관점</t>
+    </r>
     <r>
       <rPr>
         <b val="true"/>
         <sz val="11"/>
         <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">핵심 내용</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">설계 관점</t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
         <rFont val="Arial"/>
         <family val="0"/>
         <charset val="1"/>
@@ -1236,7 +1356,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">모터</t>
+      <t xml:space="preserve">차량</t>
     </r>
     <r>
       <rPr>
@@ -1255,8 +1375,20 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">로터</t>
-    </r>
+      <t xml:space="preserve">연료전지</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">WO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE</t>
   </si>
   <si>
     <r>
@@ -1266,7 +1398,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">차량</t>
+      <t xml:space="preserve">제어</t>
     </r>
     <r>
       <rPr>
@@ -1285,50 +1417,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">연료전지</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">WO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JP</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제어</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">서지</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">CN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DE</t>
   </si>
   <si>
     <r>
@@ -2246,7 +2336,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">베어링</t>
+      <t xml:space="preserve">에어포일 베어링</t>
     </r>
     <r>
       <rPr>
@@ -2263,6 +2353,40 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">기타 베어링</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">회전체 구조</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">모터</t>
     </r>
     <r>
@@ -2272,6 +2396,40 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">냉각유로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">제어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
       <t xml:space="preserve">·</t>
     </r>
     <r>
@@ -2280,7 +2438,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">로터</t>
+      <t xml:space="preserve">서지</t>
     </r>
     <r>
       <rPr>
@@ -2297,7 +2455,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">냉각</t>
+      <t xml:space="preserve">시스템</t>
     </r>
     <r>
       <rPr>
@@ -2314,7 +2472,51 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">제어</t>
+      <t xml:space="preserve">기타</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 적절한지</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  ※ 중점 분야</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">에어포일 베어링</t>
     </r>
     <r>
       <rPr>
@@ -2331,33 +2533,67 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">서지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시스템</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
+      <t xml:space="preserve">회전체 구조</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">냉각유로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 업체 외 출원인 특허도 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
     </r>
     <r>
       <rPr>
@@ -2374,15 +2610,24 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">가 적절한지</t>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">업체로 포함됩니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
     </r>
   </si>
   <si>
@@ -2643,7 +2888,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2725,6 +2970,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3033,11 +3282,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3073,16 +3322,22 @@
       <c r="I3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,B$3)</f>
@@ -3116,18 +3371,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J4" s="7" t="n">
-        <f aca="false">SUM(B4:I4)</f>
+      <c r="J4" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <f aca="false">SUM(B4:K4)</f>
         <v>1</v>
       </c>
-      <c r="K4" s="7" t="n">
+      <c r="M4" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A4,특허목록!$N:$N,"상")</f>
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B5" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$J:$J,B$3)</f>
@@ -3161,18 +3424,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J5" s="7" t="n">
-        <f aca="false">SUM(B5:I5)</f>
-        <v>0</v>
-      </c>
-      <c r="K5" s="7" t="n">
+      <c r="J5" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">SUM(B5:K5)</f>
+        <v>0</v>
+      </c>
+      <c r="M5" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A5,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A6,특허목록!$J:$J,B$3)</f>
@@ -3206,18 +3477,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A6,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="7" t="n">
-        <f aca="false">SUM(B6:I6)</f>
-        <v>0</v>
-      </c>
-      <c r="K6" s="7" t="n">
+      <c r="J6" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A6,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A6,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">SUM(B6:K6)</f>
+        <v>0</v>
+      </c>
+      <c r="M6" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A6,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A7,특허목록!$J:$J,B$3)</f>
@@ -3251,18 +3530,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A7,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="7" t="n">
-        <f aca="false">SUM(B7:I7)</f>
-        <v>0</v>
-      </c>
-      <c r="K7" s="7" t="n">
+      <c r="J7" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A7,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A7,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">SUM(B7:K7)</f>
+        <v>0</v>
+      </c>
+      <c r="M7" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A7,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,B$3)</f>
@@ -3296,18 +3583,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J8" s="7" t="n">
-        <f aca="false">SUM(B8:I8)</f>
-        <v>0</v>
-      </c>
-      <c r="K8" s="7" t="n">
+      <c r="J8" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">SUM(B8:K8)</f>
+        <v>0</v>
+      </c>
+      <c r="M8" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A8,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A9,특허목록!$J:$J,B$3)</f>
@@ -3341,18 +3636,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A9,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="7" t="n">
-        <f aca="false">SUM(B9:I9)</f>
-        <v>0</v>
-      </c>
-      <c r="K9" s="7" t="n">
+      <c r="J9" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A9,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A9,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">SUM(B9:K9)</f>
+        <v>0</v>
+      </c>
+      <c r="M9" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A9,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A10,특허목록!$J:$J,B$3)</f>
@@ -3386,18 +3689,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A10,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J10" s="7" t="n">
-        <f aca="false">SUM(B10:I10)</f>
-        <v>0</v>
-      </c>
-      <c r="K10" s="7" t="n">
+      <c r="J10" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A10,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A10,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">SUM(B10:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A10,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B11" s="6" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,B$3)</f>
@@ -3431,18 +3742,26 @@
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,I$3)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <f aca="false">SUM(B11:I11)</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="7" t="n">
+      <c r="J11" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,J$3)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$J:$J,K$3)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">SUM(B11:K11)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="7" t="n">
         <f aca="false">COUNTIFS(특허목록!$B:$B,$A11,특허목록!$N:$N,"상")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B12" s="10" t="n">
         <f aca="false">SUM(B4:B11)</f>
@@ -3478,10 +3797,18 @@
       </c>
       <c r="J12" s="10" t="n">
         <f aca="false">SUM(J4:J11)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K12" s="10" t="n">
         <f aca="false">SUM(K4:K11)</f>
+        <v>0</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <f aca="false">SUM(L4:L11)</f>
+        <v>1</v>
+      </c>
+      <c r="M12" s="10" t="n">
+        <f aca="false">SUM(M4:M11)</f>
         <v>1</v>
       </c>
     </row>
@@ -3522,93 +3849,93 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N1" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K2" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L2" s="13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M2" s="13" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N2" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O2" s="13"/>
     </row>
@@ -7020,7 +7347,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J2:J202" type="list">
-      <formula1>목록!$B$1:$B$8</formula1>
+      <formula1>목록!$B$1:$B$10</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N202" type="list">
@@ -7057,100 +7384,100 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B1" s="17" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D1" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="0" t="s">
         <v>38</v>
-      </c>
-      <c r="E1" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B3" s="17" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>6</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="F6" s="0" t="s">
         <v>62</v>
@@ -7158,7 +7485,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>8</v>
@@ -7169,13 +7496,23 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>9</v>
+        <v>64</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="17" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -7194,7 +7531,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
@@ -7202,7 +7539,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7210,17 +7547,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7228,17 +7565,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7246,7 +7583,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7254,12 +7591,12 @@
     </row>
     <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7267,22 +7604,27 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="18" t="s">
-        <v>77</v>
+      <c r="A19" s="21" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>